<commit_message>
feat(log_collector): Excel B列にTrackID専用列を追加 (SHI-38)
同一TrackIDのERROR再検知はインシデント検出済みとして扱われるが、
概要文からの正規表現抽出のみでは列としての一意キーがなかったため、
インシデントID(A列)の直後にTrackID列(B)を新設。C列以降を後方に
シフトし、汎用log-collector-skill.js/watchdog.js/excel-io.js/
web-ui/テンプレート生成/関連ドキュメントを列位置に合わせて更新した。

- watchdog.js: B列でTrackID重複判定、addRowにTrackID追加
- excel-io.js: COLSにtrackIdを追加、B列優先でtrackId取得
- log-collection-skill.js: A~F読み取りをA~Gにシフト、B列TrackIDを
  検索語に追加 (client役app.logとservice役service.logを串刺しで
  SSH grep収集できることをE2Eで確認済み)
- web-ui.html/gen-template.js: 列見出し・colspan・autoFilterを追従

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/log_collector/auto-repair-demo/examples/incident_management_template.xlsx
+++ b/projects/log_collector/auto-repair-demo/examples/incident_management_template.xlsx
@@ -11,9 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>インシデントID</t>
+  </si>
+  <si>
+    <t>TrackID</t>
   </si>
   <si>
     <t>タイムスタンプ</t>
@@ -432,22 +435,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="60" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="7" width="40" customWidth="1"/>
-    <col min="8" max="9" width="60" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="40" customWidth="1"/>
-    <col min="12" max="12" width="22" customWidth="1"/>
+    <col min="1" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="60" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="8" width="40" customWidth="1"/>
+    <col min="9" max="10" width="60" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="40" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -484,9 +487,12 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:M1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>